<commit_message>
Feat: api check existence of product name, category name. Fix: check subject condition of coupon
</commit_message>
<xml_diff>
--- a/beverage.xlsx
+++ b/beverage.xlsx
@@ -7,12 +7,16 @@
   </bookViews>
   <sheets>
     <sheet name="data" r:id="rId3" sheetId="1"/>
+    <sheet name="product" r:id="rId4" sheetId="2"/>
   </sheets>
+  <definedNames>
+    <definedName name="productName">product!$A$1:$A$2</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Product name</t>
   </si>
@@ -39,6 +43,12 @@
   </si>
   <si>
     <t>Topping price</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Product2</t>
   </si>
 </sst>
 </file>
@@ -126,14 +136,34 @@
     <dataValidation type="list" sqref="C2" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
       <formula1>"AVAILABLE,HIDDEN,OUT_OF_STOCK"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="A2" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid Value" error="Please select a valid value from the list: [A, B, C]">
-      <formula1>ISERROR(MATCH(A1, {"X","Y","Z"}, 1))</formula1>
-    </dataValidation>
     <dataValidation type="whole" operator="greaterThan" sqref="G2:G101 I2:I101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 1000." showErrorMessage="true" showInputMessage="true">
       <formula1>1000</formula1>
       <formula2>999999</formula2>
     </dataValidation>
+    <dataValidation type="custom" sqref="A2" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid Data" error="The entered value is already in the column 'stt'">
+      <formula1>COUNTIF(productName, A2)=0</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Feat: api download file import product
</commit_message>
<xml_diff>
--- a/beverage.xlsx
+++ b/beverage.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>Product name</t>
   </si>
@@ -49,6 +49,30 @@
   </si>
   <si>
     <t>Product2</t>
+  </si>
+  <si>
+    <t>Milk</t>
+  </si>
+  <si>
+    <t>Milk tea</t>
+  </si>
+  <si>
+    <t>AVAILABLE</t>
+  </si>
+  <si>
+    <t>Delicious milk tea</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/</t>
+  </si>
+  <si>
+    <t>SMALL</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>Flan</t>
   </si>
 </sst>
 </file>
@@ -93,8 +117,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="13.640625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="9.0546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="6.59375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.26171875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="6.53515625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="10.07421875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="9.46875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.8359375" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="13.2265625" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
@@ -125,22 +160,79 @@
         <v>8</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G2" t="n" s="0">
+        <v>15000.0</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="I2" t="n" s="0">
+        <v>2000.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0"/>
+      <c r="B3" s="0"/>
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="G3" t="n" s="0">
+        <v>20000.0</v>
+      </c>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0"/>
+    </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation type="list" sqref="B2" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
+  <mergeCells count="5">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+  </mergeCells>
+  <dataValidations count="6">
+    <dataValidation type="list" sqref="B2:B101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
       <formula1>"category1"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="F2" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
+    <dataValidation type="list" sqref="F2:F101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
       <formula1>"SMALL,MEDIUM,LARGE"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C2" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
+    <dataValidation type="list" sqref="C2:C101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
       <formula1>"AVAILABLE,HIDDEN,OUT_OF_STOCK"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" sqref="G2:G101 I2:I101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 1000." showErrorMessage="true" showInputMessage="true">
+    <dataValidation type="whole" operator="greaterThan" sqref="G2:G101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 1000." showErrorMessage="true" showInputMessage="true">
       <formula1>1000</formula1>
-      <formula2>999999</formula2>
-    </dataValidation>
-    <dataValidation type="custom" sqref="A2" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid Data" error="The entered value is already in the column 'stt'">
+      <formula2>9999999</formula2>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThan" sqref="I2:I101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 1000." showErrorMessage="true" showInputMessage="true">
+      <formula1>1000</formula1>
+      <formula2>9999999</formula2>
+    </dataValidation>
+    <dataValidation type="custom" sqref="A2:A101" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid Data" error="The product name is already in the database">
       <formula1>COUNTIF(productName, A2)=0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix: api create product from file Response error
</commit_message>
<xml_diff>
--- a/beverage.xlsx
+++ b/beverage.xlsx
@@ -10,13 +10,13 @@
     <sheet name="product" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="productName">product!$A$1:$A$2</definedName>
+    <definedName name="productName">product!$A$1:$A$3</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Product name</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t>Product2</t>
+  </si>
+  <si>
+    <t>Cinnamon cone</t>
   </si>
   <si>
     <t>Milk</t>
@@ -162,28 +165,28 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" t="n" s="0">
         <v>15000.0</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2" t="n" s="0">
         <v>2000.0</v>
@@ -194,11 +197,9 @@
       <c r="B3" s="0"/>
       <c r="C3" s="0"/>
       <c r="D3" s="0"/>
-      <c r="E3" t="s" s="0">
-        <v>15</v>
-      </c>
+      <c r="E3" s="0"/>
       <c r="F3" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" t="n" s="0">
         <v>20000.0</v>
@@ -224,12 +225,12 @@
     <dataValidation type="list" sqref="C2:C101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Please select a value from the drop-down list." showErrorMessage="true" showInputMessage="true" showDropDown="false">
       <formula1>"AVAILABLE,HIDDEN,OUT_OF_STOCK"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" sqref="G2:G101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 1000." showErrorMessage="true" showInputMessage="true">
-      <formula1>1000</formula1>
+    <dataValidation type="whole" operator="greaterThan" sqref="G2:G101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 999." showErrorMessage="true" showInputMessage="true">
+      <formula1>999</formula1>
       <formula2>9999999</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" sqref="I2:I101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 1000." showErrorMessage="true" showInputMessage="true">
-      <formula1>1000</formula1>
+    <dataValidation type="whole" operator="greaterThan" sqref="I2:I101" allowBlank="true" errorStyle="stop" errorTitle="Invalid Data" error="Price must be greater than 999." showErrorMessage="true" showInputMessage="true">
+      <formula1>999</formula1>
       <formula2>9999999</formula2>
     </dataValidation>
     <dataValidation type="custom" sqref="A2:A101" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid Data" error="The product name is already in the database">
@@ -242,7 +243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -255,6 +256,11 @@
         <v>10</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>